<commit_message>
Rename column to Hiring Stage (Phone Screen / Interview)
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/projects/interview-feedback-daily/Interview_Feedback_Tracker.xlsx
+++ b/projects/interview-feedback-daily/Interview_Feedback_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\claricewang\automation-learning\projects\interview-feedback-daily\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F45DF91B-A208-4A9C-8755-1F0E0E1AABA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14385E80-2BC1-4C70-BF04-B6419B095533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1808" yWindow="1808" windowWidth="16199" windowHeight="9944" xr2:uid="{D40C6D14-A354-4E8B-8970-9AD6B3527FE7}"/>
   </bookViews>
@@ -56,9 +56,6 @@
     <t>Candidate Name</t>
   </si>
   <si>
-    <t>Interview Type</t>
-  </si>
-  <si>
     <t>Interviewer</t>
   </si>
   <si>
@@ -102,6 +99,9 @@
   </si>
   <si>
     <t>Outstanding PhD, graph algo expert, suggest hire</t>
+  </si>
+  <si>
+    <t>Hiring Stage</t>
   </si>
 </sst>
 </file>
@@ -527,19 +527,19 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.45">
@@ -547,72 +547,78 @@
         <v>200034822</v>
       </c>
       <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" s="3" t="s">
         <v>13</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>14</v>
       </c>
       <c r="H2" s="2">
         <v>46125</v>
       </c>
       <c r="I2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="D3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
         <v>16</v>
       </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H3" s="2">
         <v>46125</v>
       </c>
       <c r="I3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="D4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>13</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>14</v>
       </c>
       <c r="H4" s="2">
         <v>46125</v>
       </c>
       <c r="I4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I1" xr:uid="{008E91FB-7B2A-4F0E-B7FC-C1DE26DA17E6}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{f42aa342-8706-4288-bd11-ebb85995028c}" enabled="1" method="Standard" siteId="{72f988bf-86f1-41af-91ab-2d7cd011db47}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>